<commit_message>
Inverti partite #18 e #22
https://claude.ai/code/session_017R3Evn15qdKe94BTkosKLz
</commit_message>
<xml_diff>
--- a/torneo_programma.xlsx
+++ b/torneo_programma.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programma" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classifiche" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gironi &amp; Squadre" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impianti" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cerimonie" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Programma" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Classifiche" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gironi &amp; Squadre" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Impianti" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Cerimonie" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>Dany Basket</t>
+          <t>Basket Marsciano</t>
         </is>
       </c>
       <c r="H26" s="9" t="inlineStr">
@@ -1659,12 +1659,12 @@
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>Mens Sana Siena</t>
+          <t>Endas Pistoia</t>
         </is>
       </c>
       <c r="J26" s="8" t="inlineStr">
         <is>
-          <t>Girone B13</t>
+          <t>Girone A13</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>Basket Marsciano</t>
+          <t>Dany Basket</t>
         </is>
       </c>
       <c r="H30" s="9" t="inlineStr">
@@ -1859,12 +1859,12 @@
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>Endas Pistoia</t>
+          <t>Mens Sana Siena</t>
         </is>
       </c>
       <c r="J30" s="8" t="inlineStr">
         <is>
-          <t>Girone A13</t>
+          <t>Girone B13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inverti partite #17 e #23 nella JSON sorgente
Il commit precedente a368221 aveva modificato solo index.html, lasciando
la JSON con i dati originali: la prossima rigenerazione avrebbe annullato
lo swap. Aggiorna dati_torneo.json (sorgente unico) e rigenera HTML e XLSX.

https://claude.ai/code/session_017R3Evn15qdKe94BTkosKLz
</commit_message>
<xml_diff>
--- a/torneo_programma.xlsx
+++ b/torneo_programma.xlsx
@@ -1599,7 +1599,7 @@
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>Shoemakers</t>
+          <t>Codigoro Basket</t>
         </is>
       </c>
       <c r="H25" s="9" t="inlineStr">
@@ -1609,12 +1609,12 @@
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>TissIttiri</t>
+          <t>Prato Dragons</t>
         </is>
       </c>
       <c r="J25" s="8" t="inlineStr">
         <is>
-          <t>Girone A13</t>
+          <t>Girone B13</t>
         </is>
       </c>
     </row>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>Codigoro Basket</t>
+          <t>Shoemakers</t>
         </is>
       </c>
       <c r="H31" s="9" t="inlineStr">
@@ -1909,12 +1909,12 @@
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>Prato Dragons</t>
+          <t>TissIttiri</t>
         </is>
       </c>
       <c r="J31" s="8" t="inlineStr">
         <is>
-          <t>Girone B13</t>
+          <t>Girone A13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sposta il programma pranzi nel JSON sorgente
Aggiunge la sezione "mensa" in dati_torneo.json con info_box,
slot_badges (per i badge nei riquadri partite) e giorni[].turni[]
(con fonte_partite per auto-derivazione o voci esplicite per le finali G3).

genera.py:
 - Legge i badge slot programma da mensa.slot_badges (era hardcoded)
 - Genera la sezione Mensa HTML iterando dati['mensa']['giorni']
 - Aggiunge un nuovo foglio "Mensa" all'Excel con turni e squadre

https://claude.ai/code/session_017R3Evn15qdKe94BTkosKLz
</commit_message>
<xml_diff>
--- a/torneo_programma.xlsx
+++ b/torneo_programma.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Gironi &amp; Squadre" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Impianti" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Cerimonie" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Mensa" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -104,8 +105,14 @@
       <color rgb="00166534"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -152,6 +159,21 @@
         <fgColor rgb="00EFFAE8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEDD5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -179,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -267,6 +289,18 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4209,4 +4243,910 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PROGRAMMA PRANZI</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ Schema in revisione (4 turni × 45 min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Turno</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Cat.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Squadra / Voce</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Provenienza</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GIORNO 1 — Venerdì 1 Maggio</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🟢 Turno 13:00 · 8 squadre</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Dany Basket</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>🏟 PalaCardelli 10:00</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Prato Dragons</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>🏟 PalaCardelli 10:00</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Shoemakers</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Cintolese 10:00</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Endas Pistoia</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Cintolese 10:00</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Basket Calcinaia</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Salutati 10:00</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr"/>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Massa e Cozzile</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Salutati 10:00</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr"/>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Cestistica Pescia</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Geodetica 10:00</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr"/>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Chiesina Basket</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Geodetica 10:00</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🟠 Turno 14:00 · ✈ fuori regione</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr"/>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Codigoro Basket</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>🏟 PalaCardelli 12:00</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr"/>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Mens Sana Siena</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>🏟 PalaCardelli 12:00</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr"/>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Basket Marsciano</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Cintolese 12:00</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>TissIttiri</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Cintolese 12:00</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr"/>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Basket Loano</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Salutati 12:00</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr"/>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Shoemakers</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Salutati 12:00</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr"/>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>La T Gema</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Geodetica 12:00</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr"/>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>San Fr. Ittiri</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Geodetica 12:00</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GIORNO 2 — Sabato 2 Maggio</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🟢 Turno 12:00 · 8 squadre</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr"/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Codigoro Basket</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>🏟 PalaCardelli 09:00</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr"/>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Prato Dragons</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>🏟 PalaCardelli 09:00</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr"/>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Basket Marsciano</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Cintolese 09:00</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr"/>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Endas Pistoia</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Cintolese 09:00</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr"/>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Massa e Cozzile</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Salutati 09:00</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr"/>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Shoemakers</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Salutati 09:00</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr"/>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Cestistica Pescia</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Geodetica 09:00</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr"/>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>La T Gema</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Geodetica 09:00</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🟠 Turno 13:00 · 8 squadre</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr"/>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Basket Calcinaia</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>🏟 PalaCardelli 11:00</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr"/>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Basket Loano</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>🏟 PalaCardelli 11:00</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr"/>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Dany Basket</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Cintolese 11:00</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr"/>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Mens Sana Siena</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Cintolese 11:00</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr"/>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Shoemakers</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Salutati 11:00</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr"/>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>TissIttiri</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Salutati 11:00</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr"/>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Chiesina Basket</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Geodetica 11:00</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr"/>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>San Fr. Ittiri</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Geodetica 11:00</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GIORNO 3 — Domenica 3 Maggio</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🟢 Turno 12:00 · finali mattutine U13</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr"/>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Finale 3°/4°</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Pala 09:00</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr"/>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Finale 5°/6°</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Geodetica 09:00</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr"/>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Finale 7°/8°</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Cintolese 09:00</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🟠 Turno 13:00 · prima delle finalissime</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr"/>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Finale 3°/4°</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Pala 11:00</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr"/>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>Finale 5°/6°</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Geodetica 11:00</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr"/>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>Finale 7°/8°</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Cintolese 11:00</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr"/>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>🏆 Finaliste U13</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>(prima della finale)</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🟡 Turno 14:30 · finaliste U14</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr"/>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>🏆 Finaliste U14</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>(prima della finale 15:00)</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Aggiungi Caffè Micky come punto di ristoro per Cintolese
https://claude.ai/code/session_017R3Evn15qdKe94BTkosKLz
</commit_message>
<xml_diff>
--- a/torneo_programma.xlsx
+++ b/torneo_programma.xlsx
@@ -3955,7 +3955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4134,6 +4134,33 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>☕</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Caffè Micky</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>Cintolese · Monsummano Terme</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>Punto di ristoro ufficiale per i pranzi delle squadre che giocano alla Pal. Cintolese.</t>
+        </is>
+      </c>
+      <c r="E9" s="28" t="inlineStr">
+        <is>
+          <t>📍 Apri su Maps</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
@@ -4144,6 +4171,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Aggiorna griglia pranzi da Excel: orari, PAX, allergie, locali
- dati_torneo.json: mensa ricostruita con dati reali (orari corretti 12:30/13:30/14:00,
  PAX per squadra, allergie/intolleranze, suddivisione per locale Caffè Micky / Pool Bar)
- slot_badges aggiornati con orari corretti
- genera.py: turno_items e turno_list_html renderizzano pax e allergie;
  foglio Excel mensa aggiornato con colonne PAX e Allergie

https://claude.ai/code/session_01L71tgdEaT7WMMAgsiZmcki
</commit_message>
<xml_diff>
--- a/torneo_programma.xlsx
+++ b/torneo_programma.xlsx
@@ -290,8 +290,8 @@
     <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4270,7 +4270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4300,17 +4300,17 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Squadra / Voce</t>
+          <t>Squadra</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Provenienza</t>
+          <t>PAX</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>Allergie &amp; intolleranze</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
     <row r="5">
       <c r="A5" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🟢 Turno 13:00 · 8 squadre</t>
+          <t xml:space="preserve">  ☕ Caffè Micky · 12:30 · 24 coperti</t>
         </is>
       </c>
     </row>
@@ -4337,53 +4337,45 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Dany Basket</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>🏟 PalaCardelli 10:00</t>
+          <t>Endas Pistoia</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>24 pax</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr"/>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Prato Dragons</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>🏟 PalaCardelli 10:00</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr"/>
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🍽 Pool Bar · 12:30 · 25 coperti · ⚠ allergie</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Shoemakers</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Cintolese 10:00</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr"/>
+          <t>Chiesina Basket</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>15 pax</t>
+        </is>
+      </c>
+      <c r="E8" s="32" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr"/>
@@ -4394,88 +4386,84 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Endas Pistoia</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Cintolese 10:00</t>
+          <t>Dany Basket</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>10 pax</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Basket Calcinaia</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Salutati 10:00</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr"/>
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ☕ Caffè Micky · 14:00 · 76 coperti · ⚠ allergie</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Massa e Cozzile</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Salutati 10:00</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr"/>
+          <t>Mens Sana Siena</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>36 pax</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Fucecchio</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Geodetica 10:00</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr"/>
+          <t>TissIttiri</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>24 pax</t>
+        </is>
+      </c>
+      <c r="E12" s="32" t="inlineStr">
+        <is>
+          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Chiesina Basket</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Geodetica 10:00</t>
+          <t>Basket Marsciano</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>16 pax</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr"/>
@@ -4483,7 +4471,7 @@
     <row r="14">
       <c r="A14" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🟠 Turno 14:00 · ✈ fuori regione</t>
+          <t xml:space="preserve">  🍽 Pool Bar · 14:00 · 65 coperti · ⚠ allergie</t>
         </is>
       </c>
     </row>
@@ -4499,178 +4487,154 @@
           <t>Codigoro Basket</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>🏟 PalaCardelli 12:00</t>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>35 pax</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr"/>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Mens Sana Siena</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>🏟 PalaCardelli 12:00</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr"/>
+          <t>Basket Loano</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>18 pax</t>
+        </is>
+      </c>
+      <c r="E16" s="32" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr"/>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Basket Marsciano</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Cintolese 12:00</t>
+          <t>San Fr. Ittiri</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>12 pax</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr"/>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr"/>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>TissIttiri</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Cintolese 12:00</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr"/>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Basket Loano</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Salutati 12:00</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr"/>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GIORNO 2 — Sabato 2 Maggio</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr"/>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Shoemakers</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Salutati 12:00</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr"/>
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ☕ Caffè Micky · 12:30 · 16 coperti</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr"/>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>La T Gema</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>Geodetica 12:00</t>
+          <t>Basket Marsciano</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>16 pax</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr"/>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>San Fr. Ittiri</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Geodetica 12:00</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr"/>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  GIORNO 2 — Sabato 2 Maggio</t>
+      <c r="A22" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🍽 Pool Bar · 12:30 · 24 coperti · ⚠ allergie</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr"/>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>TissIttiri</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>24 pax</t>
+        </is>
+      </c>
+      <c r="E23" s="32" t="inlineStr">
+        <is>
+          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ☕ Caffè Micky · 13:30 · 4 coperti · ⚠ allergie</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🟢 Turno 12:00 · 8 squadre</t>
+      <c r="A25" s="5" t="inlineStr"/>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Mens Sana Siena</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>4 pax</t>
+        </is>
+      </c>
+      <c r="E25" s="32" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr"/>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Codigoro Basket</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>🏟 PalaCardelli 09:00</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr"/>
+      <c r="A26" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🍽 Pool Bar · 13:30 · 80 coperti · ⚠ allergie</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr"/>
@@ -4681,53 +4645,61 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Prato Dragons</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>🏟 PalaCardelli 09:00</t>
+          <t>Codigoro Basket</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>35 pax</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr"/>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Basket Marsciano</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Cintolese 09:00</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr"/>
+          <t>Basket Loano</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>18 pax</t>
+        </is>
+      </c>
+      <c r="E28" s="32" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr"/>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Endas Pistoia</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>Cintolese 09:00</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="inlineStr"/>
+          <t>Chiesina Basket</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>15 pax</t>
+        </is>
+      </c>
+      <c r="E29" s="32" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr"/>
@@ -4738,98 +4710,71 @@
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>Massa e Cozzile</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Salutati 09:00</t>
+          <t>San Fr. Ittiri</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>12 pax</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr"/>
     </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr"/>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Shoemakers</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>Salutati 09:00</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr"/>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Fucecchio</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>Geodetica 09:00</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr"/>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GIORNO 3 — Domenica 3 Maggio</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr"/>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>La T Gema</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>Geodetica 09:00</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr"/>
+      <c r="A33" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🍽 Pool Bar · 14:00 · 120 coperti · ⚠ allergie</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🟠 Turno 13:00 · 8 squadre</t>
-        </is>
-      </c>
+      <c r="A34" s="5" t="inlineStr"/>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Codigoro Basket</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>35 pax</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr"/>
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Basket Calcinaia</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>🏟 PalaCardelli 11:00</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr"/>
+          <t>TissIttiri</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>24 pax</t>
+        </is>
+      </c>
+      <c r="E35" s="32" t="inlineStr">
+        <is>
+          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr"/>
@@ -4843,12 +4788,16 @@
           <t>Basket Loano</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>🏟 PalaCardelli 11:00</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr"/>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>18 pax</t>
+        </is>
+      </c>
+      <c r="E36" s="32" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr"/>
@@ -4859,304 +4808,73 @@
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Dany Basket</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>Cintolese 11:00</t>
+          <t>Basket Marsciano</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>16 pax</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr"/>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Mens Sana Siena</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Cintolese 11:00</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr"/>
+          <t>Chiesina Basket</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>15 pax</t>
+        </is>
+      </c>
+      <c r="E38" s="32" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr"/>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Shoemakers</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Salutati 11:00</t>
+          <t>San Fr. Ittiri</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>12 pax</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr"/>
     </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr"/>
-      <c r="B40" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>TissIttiri</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>Salutati 11:00</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr"/>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>Chiesina Basket</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Geodetica 11:00</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr"/>
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>San Fr. Ittiri</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Geodetica 11:00</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr"/>
-    </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  GIORNO 3 — Domenica 3 Maggio</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🟢 Turno 12:00 · finali mattutine U13</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr"/>
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>Finale 3°/4°</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>Pala 09:00</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr"/>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>Finale 5°/6°</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>Geodetica 09:00</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr"/>
-      <c r="B48" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>Finale 7°/8°</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>Cintolese 09:00</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🟠 Turno 13:00 · prima delle finalissime</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr"/>
-      <c r="B50" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>Finale 3°/4°</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Pala 11:00</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr"/>
-      <c r="B51" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>Finale 5°/6°</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Geodetica 11:00</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr"/>
-      <c r="B52" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>Finale 7°/8°</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Cintolese 11:00</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr"/>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>🏆 Finaliste U13</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>(prima della finale)</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🟡 Turno 14:30 · finaliste U14</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr"/>
-      <c r="B55" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>🏆 Finaliste U14</t>
-        </is>
-      </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>(prima della finale 15:00)</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr"/>
-    </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A34:E34"/>
+  <mergeCells count="13">
     <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A54:E54"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A33:E33"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A32:E32"/>
     <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A22:E22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Corregge pranzo Mens Sana Siena: Caffè Micky → Pool Bar (ven 14:00)
https://claude.ai/code/session_01L71tgdEaT7WMMAgsiZmcki
</commit_message>
<xml_diff>
--- a/torneo_programma.xlsx
+++ b/torneo_programma.xlsx
@@ -4399,7 +4399,7 @@
     <row r="10">
       <c r="A10" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ☕ Caffè Micky · 14:00 · 76 coperti · ⚠ allergie</t>
+          <t xml:space="preserve">  ☕ Caffè Micky · 14:00 · 40 coperti · ⚠ allergie</t>
         </is>
       </c>
     </row>
@@ -4412,17 +4412,17 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Mens Sana Siena</t>
+          <t>TissIttiri</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>36 pax</t>
+          <t>24 pax</t>
         </is>
       </c>
       <c r="E11" s="32" t="inlineStr">
         <is>
-          <t>⚠ 1 celiaco</t>
+          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
         </is>
       </c>
     </row>
@@ -4435,43 +4435,43 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>TissIttiri</t>
+          <t>Basket Marsciano</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>24 pax</t>
-        </is>
-      </c>
-      <c r="E12" s="32" t="inlineStr">
-        <is>
-          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
-        </is>
-      </c>
+          <t>16 pax</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr"/>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🍽 Pool Bar · 14:00 · 101 coperti · ⚠ allergie</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>U13</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Basket Marsciano</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>16 pax</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🍽 Pool Bar · 14:00 · 65 coperti · ⚠ allergie</t>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Mens Sana Siena</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>36 pax</t>
+        </is>
+      </c>
+      <c r="E14" s="32" t="inlineStr">
+        <is>
+          <t>⚠ 1 celiaco</t>
         </is>
       </c>
     </row>
@@ -4873,7 +4873,7 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A13:E13"/>
     <mergeCell ref="A22:E22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Nasconde mensa Domenica da HTML e Excel (da confermare)
https://claude.ai/code/session_01L71tgdEaT7WMMAgsiZmcki
</commit_message>
<xml_diff>
--- a/torneo_programma.xlsx
+++ b/torneo_programma.xlsx
@@ -4270,7 +4270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4720,148 +4720,8 @@
       </c>
       <c r="E30" s="8" t="inlineStr"/>
     </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  GIORNO 3 — Domenica 3 Maggio</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🍽 Pool Bar · 14:00 · 120 coperti · ⚠ allergie</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr"/>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>Codigoro Basket</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>35 pax</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr"/>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>TissIttiri</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>24 pax</t>
-        </is>
-      </c>
-      <c r="E35" s="32" t="inlineStr">
-        <is>
-          <t>⚠ allergia peperoncino · intolleranza lattosio · allergia tonno</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr"/>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>Basket Loano</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>18 pax</t>
-        </is>
-      </c>
-      <c r="E36" s="32" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr"/>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>Basket Marsciano</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>16 pax</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr"/>
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>Chiesina Basket</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>15 pax</t>
-        </is>
-      </c>
-      <c r="E38" s="32" t="inlineStr">
-        <is>
-          <t>⚠ 1 celiaco · 1 intollerante lattosio</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr"/>
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>San Fr. Ittiri</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>12 pax</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr"/>
-    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="11">
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="A24:E24"/>
@@ -4869,10 +4729,8 @@
     <mergeCell ref="A7:E7"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A33:E33"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A32:E32"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A22:E22"/>
   </mergeCells>

</xml_diff>

<commit_message>
Programma Domenica 3 Maggio (G3): finali e mini-torneo U14 a Cintolese
- F3/4 U13 (PalaCardelli 11:00): Codigoro vs Marsciano
- F7/8 U13 (Geodetica 09:00): Endas Pistoia vs Dany Basket
- F5/6 U13 (Geodetica 11:00): Mens Sana vs TissIttiri
- F3/4 U14 (PalaCardelli 09:00): La T Gema vs Chiesina
- Finalissima U13 (PalaCardelli 13:00): Shoemakers vs Prato Dragons
- Finalissima U14 (PalaCardelli 15:00): Shoemakers vs Calcinaia
- Massa e Cozzile rinuncia: mini-torneo 5°-7° U14 a Cintolese
  (Fucecchio-Loano 10:00, Fucecchio-S.Fr.Ittiri 10:45, Loano-S.Fr.Ittiri 11:30)
</commit_message>
<xml_diff>
--- a/torneo_programma.xlsx
+++ b/torneo_programma.xlsx
@@ -666,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2432,29 +2432,29 @@
           <t>🏟 PalaCardelli</t>
         </is>
       </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
         </is>
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>Perd.SF-Oro1</t>
+          <t>La T Gema</t>
         </is>
       </c>
       <c r="H43" s="15" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>0 – 0</t>
         </is>
       </c>
       <c r="I43" s="8" t="inlineStr">
         <is>
-          <t>Perd.SF-Oro2</t>
+          <t>Chiesina Basket</t>
         </is>
       </c>
       <c r="J43" s="14" t="inlineStr">
         <is>
-          <t>Finale 3°/4° U13</t>
+          <t>Finale 3°/4° U14</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Pal. Cintolese</t>
+          <t>Geodetica</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
@@ -2489,17 +2489,17 @@
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>Perd.SF-Bronzo1</t>
+          <t>Endas Pistoia</t>
         </is>
       </c>
       <c r="H44" s="15" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>0 – 0</t>
         </is>
       </c>
       <c r="I44" s="8" t="inlineStr">
         <is>
-          <t>Perd.SF-Bronzo2</t>
+          <t>Dany Basket</t>
         </is>
       </c>
       <c r="J44" s="14" t="inlineStr">
@@ -2524,37 +2524,37 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Geodetica</t>
-        </is>
-      </c>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
+          <t>Pal. Cintolese</t>
+        </is>
+      </c>
+      <c r="F45" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>Vinc.SF-Bronzo1</t>
+          <t>Fucecchio</t>
         </is>
       </c>
       <c r="H45" s="15" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>0 – 0</t>
         </is>
       </c>
       <c r="I45" s="8" t="inlineStr">
         <is>
-          <t>Vinc.SF-Bronzo2</t>
-        </is>
-      </c>
-      <c r="J45" s="14" t="inlineStr">
-        <is>
-          <t>Finale 5°/6° U13</t>
+          <t>Basket Loano</t>
+        </is>
+      </c>
+      <c r="J45" s="8" t="inlineStr">
+        <is>
+          <t>Mini-torneo 5°-7° U14</t>
         </is>
       </c>
     </row>
@@ -2574,12 +2574,12 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>🏟 PalaCardelli</t>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Pal. Cintolese</t>
         </is>
       </c>
       <c r="F46" s="10" t="inlineStr">
@@ -2589,22 +2589,22 @@
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>Perd.SF-Oro1</t>
+          <t>Fucecchio</t>
         </is>
       </c>
       <c r="H46" s="15" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>0 – 0</t>
         </is>
       </c>
       <c r="I46" s="8" t="inlineStr">
         <is>
-          <t>Perd.SF-Oro2</t>
-        </is>
-      </c>
-      <c r="J46" s="14" t="inlineStr">
-        <is>
-          <t>Finale 3°/4° U14</t>
+          <t>San Fr. Ittiri</t>
+        </is>
+      </c>
+      <c r="J46" s="8" t="inlineStr">
+        <is>
+          <t>Mini-torneo 5°-7° U14</t>
         </is>
       </c>
     </row>
@@ -2627,34 +2627,34 @@
           <t>11:00</t>
         </is>
       </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Pal. Cintolese</t>
-        </is>
-      </c>
-      <c r="F47" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>🏟 PalaCardelli</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
         </is>
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>Perd.SF-Bronzo1</t>
+          <t>Codigoro Basket</t>
         </is>
       </c>
       <c r="H47" s="15" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>0 – 0</t>
         </is>
       </c>
       <c r="I47" s="8" t="inlineStr">
         <is>
-          <t>Perd.SF-Bronzo2</t>
+          <t>Basket Marsciano</t>
         </is>
       </c>
       <c r="J47" s="14" t="inlineStr">
         <is>
-          <t>Finale 7°/8° U14</t>
+          <t>Finale 3°/4° U13</t>
         </is>
       </c>
     </row>
@@ -2682,29 +2682,29 @@
           <t>Geodetica</t>
         </is>
       </c>
-      <c r="F48" s="10" t="inlineStr">
-        <is>
-          <t>U14</t>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>Vinc.SF-Bronzo1</t>
+          <t>Mens Sana Siena</t>
         </is>
       </c>
       <c r="H48" s="15" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>0 – 0</t>
         </is>
       </c>
       <c r="I48" s="8" t="inlineStr">
         <is>
-          <t>Vinc.SF-Bronzo2</t>
+          <t>TissIttiri</t>
         </is>
       </c>
       <c r="J48" s="14" t="inlineStr">
         <is>
-          <t>Finale 5°/6° U14</t>
+          <t>Finale 5°/6° U13</t>
         </is>
       </c>
     </row>
@@ -2724,37 +2724,37 @@
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="E49" s="6" t="inlineStr">
-        <is>
-          <t>🏟 PalaCardelli</t>
-        </is>
-      </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="G49" s="16" t="inlineStr">
-        <is>
-          <t>Vinc.SF-Oro1</t>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Pal. Cintolese</t>
+        </is>
+      </c>
+      <c r="F49" s="10" t="inlineStr">
+        <is>
+          <t>U14</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>Basket Loano</t>
         </is>
       </c>
       <c r="H49" s="15" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>0 – 0</t>
         </is>
       </c>
       <c r="I49" s="8" t="inlineStr">
         <is>
-          <t>Vinc.SF-Oro2</t>
-        </is>
-      </c>
-      <c r="J49" s="14" t="inlineStr">
-        <is>
-          <t>🏆 FINALISSIMA 1°/2° U13</t>
+          <t>San Fr. Ittiri</t>
+        </is>
+      </c>
+      <c r="J49" s="8" t="inlineStr">
+        <is>
+          <t>Mini-torneo 5°-7° U14</t>
         </is>
       </c>
     </row>
@@ -2774,75 +2774,125 @@
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>🏟 PalaCardelli</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="G50" s="16" t="inlineStr">
+        <is>
+          <t>Shoemakers</t>
+        </is>
+      </c>
+      <c r="H50" s="15" t="inlineStr">
+        <is>
+          <t>0 – 0</t>
+        </is>
+      </c>
+      <c r="I50" s="8" t="inlineStr">
+        <is>
+          <t>Prato Dragons</t>
+        </is>
+      </c>
+      <c r="J50" s="14" t="inlineStr">
+        <is>
+          <t>🏆 FINALISSIMA 1°/2° U13</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Giorno 3</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Dom 3 Mag</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E51" s="6" t="inlineStr">
         <is>
           <t>🏟 PalaCardelli</t>
         </is>
       </c>
-      <c r="F50" s="10" t="inlineStr">
+      <c r="F51" s="10" t="inlineStr">
         <is>
           <t>U14</t>
         </is>
       </c>
-      <c r="G50" s="16" t="inlineStr">
-        <is>
-          <t>Vinc.SF-Oro1</t>
-        </is>
-      </c>
-      <c r="H50" s="15" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I50" s="8" t="inlineStr">
-        <is>
-          <t>Vinc.SF-Oro2</t>
-        </is>
-      </c>
-      <c r="J50" s="14" t="inlineStr">
+      <c r="G51" s="16" t="inlineStr">
+        <is>
+          <t>Shoemakers</t>
+        </is>
+      </c>
+      <c r="H51" s="15" t="inlineStr">
+        <is>
+          <t>0 – 0</t>
+        </is>
+      </c>
+      <c r="I51" s="8" t="inlineStr">
+        <is>
+          <t>Basket Calcinaia</t>
+        </is>
+      </c>
+      <c r="J51" s="14" t="inlineStr">
         <is>
           <t>🏆 FINALISSIMA 1°/2° U14</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="11" t="inlineStr"/>
-      <c r="B51" s="11" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr"/>
+      <c r="B52" s="11" t="inlineStr">
         <is>
           <t>Giorno 3</t>
         </is>
       </c>
-      <c r="C51" s="11" t="inlineStr">
+      <c r="C52" s="11" t="inlineStr">
         <is>
           <t>Dom 3 Mag</t>
         </is>
       </c>
-      <c r="D51" s="11" t="inlineStr">
+      <c r="D52" s="11" t="inlineStr">
         <is>
           <t>17:00–17:45</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>🏟 PalaCardelli</t>
         </is>
       </c>
-      <c r="F51" s="11" t="inlineStr">
+      <c r="F52" s="11" t="inlineStr">
         <is>
           <t>TUTTI</t>
         </is>
       </c>
-      <c r="G51" s="12" t="inlineStr">
+      <c r="G52" s="12" t="inlineStr">
         <is>
           <t>CERIMONIA DI CHIUSURA</t>
         </is>
       </c>
-      <c r="H51" s="11" t="inlineStr"/>
-      <c r="I51" s="13" t="inlineStr"/>
-      <c r="J51" s="13" t="inlineStr">
+      <c r="H52" s="11" t="inlineStr"/>
+      <c r="I52" s="13" t="inlineStr"/>
+      <c r="J52" s="13" t="inlineStr">
         <is>
           <t>🏆 Premiazioni di tutte le categorie</t>
         </is>

</xml_diff>

<commit_message>
Mini-torneo U14: indica durata partite (45') nella fase
Le partite del mini-torneo 5°-7° U14 hanno durata ridotta (45 minuti
invece dei tempi standard). Aggiunto '(45')' alla fase per renderlo
visibile sia su sito che su Excel.
</commit_message>
<xml_diff>
--- a/torneo_programma.xlsx
+++ b/torneo_programma.xlsx
@@ -2554,7 +2554,7 @@
       </c>
       <c r="J45" s="8" t="inlineStr">
         <is>
-          <t>Mini-torneo 5°-7° U14</t>
+          <t>Mini-torneo 5°-7° U14 (45')</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2604,7 @@
       </c>
       <c r="J46" s="8" t="inlineStr">
         <is>
-          <t>Mini-torneo 5°-7° U14</t>
+          <t>Mini-torneo 5°-7° U14 (45')</t>
         </is>
       </c>
     </row>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="J49" s="8" t="inlineStr">
         <is>
-          <t>Mini-torneo 5°-7° U14</t>
+          <t>Mini-torneo 5°-7° U14 (45')</t>
         </is>
       </c>
     </row>

</xml_diff>